<commit_message>
can we log genkit logs tto the log viewer as well
</commit_message>
<xml_diff>
--- a/public/csv_data_store/catalog.xlsx
+++ b/public/csv_data_store/catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sean1002\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6570D7-FE39-41DE-93C0-B8B5AC596F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4980EB9F-57D1-4FDC-93FD-6AF5EC5D8FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{7E2D1D46-A7F7-405F-A549-D6848E67490D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" activeTab="1" xr2:uid="{7E2D1D46-A7F7-405F-A549-D6848E67490D}"/>
   </bookViews>
   <sheets>
     <sheet name="datasets" sheetId="3" r:id="rId1"/>
@@ -1950,7 +1950,7 @@
         <v>27</v>
       </c>
       <c r="C2">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
@@ -2007,7 +2007,7 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
@@ -2064,7 +2064,7 @@
         <v>27</v>
       </c>
       <c r="C4">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -2121,7 +2121,7 @@
         <v>27</v>
       </c>
       <c r="C5">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="D5" t="s">
         <v>9</v>
@@ -2178,7 +2178,7 @@
         <v>27</v>
       </c>
       <c r="C6">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="D6" t="s">
         <v>9</v>
@@ -2235,7 +2235,7 @@
         <v>27</v>
       </c>
       <c r="C7">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D7" t="s">
         <v>4</v>
@@ -2292,7 +2292,7 @@
         <v>27</v>
       </c>
       <c r="C8">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D8" t="s">
         <v>4</v>
@@ -2349,7 +2349,7 @@
         <v>27</v>
       </c>
       <c r="C9">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D9" t="s">
         <v>4</v>
@@ -2406,7 +2406,7 @@
         <v>27</v>
       </c>
       <c r="C10">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D10" t="s">
         <v>4</v>
@@ -2463,7 +2463,7 @@
         <v>27</v>
       </c>
       <c r="C11">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D11" t="s">
         <v>4</v>
@@ -2520,7 +2520,7 @@
         <v>27</v>
       </c>
       <c r="C12">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D12" t="s">
         <v>4</v>
@@ -2577,7 +2577,7 @@
         <v>27</v>
       </c>
       <c r="C13">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D13" t="s">
         <v>4</v>
@@ -2634,7 +2634,7 @@
         <v>27</v>
       </c>
       <c r="C14">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D14" t="s">
         <v>4</v>

</xml_diff>